<commit_message>
Set owner's strip ratio (4) and mineable reserve (400,000 t)
Both remain editable input cells; excavator capacity and reserve
sufficiency checks now pass. Items-to-confirm sheet links to the inputs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018UUydQjRuPdneArnVH1qrQ
</commit_message>
<xml_diff>
--- a/chromite-quarry-feasibility/Chromite-Quarry-Feasibility-Monthly-Production.xlsx
+++ b/chromite-quarry-feasibility/Chromite-Quarry-Feasibility-Monthly-Production.xlsx
@@ -7890,7 +7890,7 @@
     <row r="35">
       <c r="A35" s="2" t="str">
         <f>"5) الحفارات: "&amp;'الخطة الفنية والإنتاج'!C14&amp;" — الاحتياطي: "&amp;'الخطة الفنية والإنتاج'!B28</f>
-        <v>5) الحفارات: غير كافية — المطلوب 155% من طاقتها؛ يلزم ألا تزيد نسبة التعرية عن 4.8 أو إنتاجية أعلى أو حفارات إضافية — الاحتياطي: تنبيه: الاحتياطي المفترض (140,000 طن) لا يكفي — المطلوب 352,941 طن خام لخمس سنوات</v>
+        <v>5) الحفارات: كافية — المطلوب 86% من طاقة الحفارات — الاحتياطي: الاحتياطي المفترض كافٍ لخمس سنوات تشغيل</v>
       </c>
     </row>
   </sheetData>
@@ -9881,10 +9881,9 @@
           <t>الاحتياطي ودرجة الخام</t>
         </is>
       </c>
-      <c r="C27" s="43" t="inlineStr">
-        <is>
-          <t>140,000 طن بدرجة 32%</t>
-        </is>
+      <c r="C27" s="43" t="str">
+        <f>TEXT(OreReserve,"#,##0")&amp;" طن بدرجة "&amp;TEXT(OreGrade,"0%")</f>
+        <v>400,000 طن بدرجة 32%</v>
       </c>
       <c r="D27" s="43" t="inlineStr">
         <is>
@@ -9905,10 +9904,9 @@
           <t>نسبة التعرية وإنتاجية التكسير</t>
         </is>
       </c>
-      <c r="C28" s="43" t="inlineStr">
-        <is>
-          <t>8 طن/طن و35 طن/ساعة</t>
-        </is>
+      <c r="C28" s="43" t="str">
+        <f>TEXT(StripRatio,"0.0")&amp;" طن/طن و"&amp;TEXT(BrkProd,"0")&amp;" طن/ساعة"</f>
+        <v>4.0 طن/طن و35 طن/ساعة</v>
       </c>
       <c r="D28" s="43" t="inlineStr">
         <is>
@@ -10512,7 +10510,7 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>140000</v>
+        <v>400000</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
@@ -10521,7 +10519,7 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>افتراض يحتاج تأكيداً — غير وارد في الملف الأصلي. يُستبدل برقم التقرير الاستكشافي المعتمد</t>
+          <t>معطى من المالك (أكتوبر 2026) — يُوثَّق بالتقرير الاستكشافي المعتمد</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10550,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
@@ -10561,7 +10559,7 @@
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>افتراض يحتاج تأكيداً — يحدد حجم الصخور المطلوب تحريكها وكفاية الحفارات</t>
+          <t>معطى من المالك (أكتوبر 2026) — يحدد حجم الصخور المطلوب تحريكها وكفاية الحفارات</t>
         </is>
       </c>
     </row>
@@ -12859,7 +12857,7 @@
       </c>
       <c r="C10" s="11">
         <f>ROMCap*(1+StripRatio)</f>
-        <v>635294.117647059</v>
+        <v>352941.176470588</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -12880,7 +12878,7 @@
       </c>
       <c r="C11" s="11">
         <f>RockCap-ROMCap</f>
-        <v>564705.882352941</v>
+        <v>282352.941176471</v>
       </c>
     </row>
     <row r="12">
@@ -12917,7 +12915,7 @@
       </c>
       <c r="C13" s="17">
         <f>IF(C12&gt;0,C10/C12,0)</f>
-        <v>1.5513897866839</v>
+        <v>0.861883214824391</v>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
@@ -12934,7 +12932,7 @@
       <c r="B14" s="22" t="n"/>
       <c r="C14" s="22" t="str">
         <f>IF(C13&lt;=1,"كافية — المطلوب "&amp;TEXT(C13,"0%")&amp;" من طاقة الحفارات","غير كافية — المطلوب "&amp;TEXT(C13,"0%")&amp;" من طاقتها؛ يلزم ألا تزيد نسبة التعرية عن "&amp;TEXT(C15,"0.0")&amp;" أو إنتاجية أعلى أو حفارات إضافية")</f>
-        <v>غير كافية — المطلوب 155% من طاقتها؛ يلزم ألا تزيد نسبة التعرية عن 4.8 أو إنتاجية أعلى أو حفارات إضافية</v>
+        <v>كافية — المطلوب 86% من طاقة الحفارات</v>
       </c>
       <c r="D14" s="22" t="n"/>
       <c r="E14" s="22" t="n"/>
@@ -12997,7 +12995,7 @@
       </c>
       <c r="C17" s="31">
         <f>IF(ROMCap&gt;0,OreReserve/ROMCap,0)</f>
-        <v>1.98333333333333</v>
+        <v>5.66666666666667</v>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
@@ -13107,27 +13105,27 @@
       </c>
       <c r="D22" s="11">
         <f>RockCap*D20</f>
-        <v>635294.117647059</v>
+        <v>352941.176470588</v>
       </c>
       <c r="E22" s="11">
         <f>RockCap*E20</f>
-        <v>635294.117647059</v>
+        <v>352941.176470588</v>
       </c>
       <c r="F22" s="11">
         <f>RockCap*F20</f>
-        <v>635294.117647059</v>
+        <v>352941.176470588</v>
       </c>
       <c r="G22" s="11">
         <f>RockCap*G20</f>
-        <v>635294.117647059</v>
+        <v>352941.176470588</v>
       </c>
       <c r="H22" s="11">
         <f>RockCap*H20</f>
-        <v>635294.117647059</v>
+        <v>352941.176470588</v>
       </c>
       <c r="I22" s="12">
         <f>SUM(D22:H22)</f>
-        <v>3176470.58823529</v>
+        <v>1764705.88235294</v>
       </c>
     </row>
     <row r="23">
@@ -13283,27 +13281,27 @@
       </c>
       <c r="C27" s="11">
         <f>OreReserve</f>
-        <v>140000</v>
+        <v>400000</v>
       </c>
       <c r="D27" s="11">
         <f>OreReserve-D26</f>
-        <v>69411.7647058824</v>
+        <v>329411.764705882</v>
       </c>
       <c r="E27" s="11">
         <f>OreReserve-E26</f>
-        <v>-1176.4705882353</v>
+        <v>258823.529411765</v>
       </c>
       <c r="F27" s="11">
         <f>OreReserve-F26</f>
-        <v>-71764.705882353</v>
+        <v>188235.294117647</v>
       </c>
       <c r="G27" s="11">
         <f>OreReserve-G26</f>
-        <v>-142352.941176471</v>
+        <v>117647.058823529</v>
       </c>
       <c r="H27" s="11">
         <f>OreReserve-H26</f>
-        <v>-212941.176470588</v>
+        <v>47058.8235294118</v>
       </c>
     </row>
     <row r="28">
@@ -13314,7 +13312,7 @@
       </c>
       <c r="B28" s="21" t="str">
         <f>IF($H$27&gt;=0,"الاحتياطي المفترض كافٍ لخمس سنوات تشغيل","تنبيه: الاحتياطي المفترض ("&amp;TEXT(OreReserve,"#,##0")&amp;" طن) لا يكفي — المطلوب "&amp;TEXT($H$26,"#,##0")&amp;" طن خام لخمس سنوات")</f>
-        <v>تنبيه: الاحتياطي المفترض (140,000 طن) لا يكفي — المطلوب 352,941 طن خام لخمس سنوات</v>
+        <v>الاحتياطي المفترض كافٍ لخمس سنوات تشغيل</v>
       </c>
       <c r="C28" s="22" t="n"/>
       <c r="D28" s="22" t="n"/>
@@ -13542,7 +13540,7 @@
       </c>
       <c r="F6" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B6)*D6/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G6" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B6)*D6/$N$18,0)</f>
@@ -13562,7 +13560,7 @@
       </c>
       <c r="K6" s="11">
         <f>OreReserve-SUM($G$6:G6)</f>
-        <v>134117.647058824</v>
+        <v>394117.647058824</v>
       </c>
       <c r="M6" s="43" t="inlineStr">
         <is>
@@ -13595,7 +13593,7 @@
       </c>
       <c r="F7" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B7)*D7/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G7" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B7)*D7/$N$18,0)</f>
@@ -13615,7 +13613,7 @@
       </c>
       <c r="K7" s="11">
         <f>OreReserve-SUM($G$6:G7)</f>
-        <v>128235.294117647</v>
+        <v>388235.294117647</v>
       </c>
       <c r="M7" s="43" t="inlineStr">
         <is>
@@ -13648,7 +13646,7 @@
       </c>
       <c r="F8" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B8)*D8/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G8" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B8)*D8/$N$18,0)</f>
@@ -13668,7 +13666,7 @@
       </c>
       <c r="K8" s="11">
         <f>OreReserve-SUM($G$6:G8)</f>
-        <v>122352.941176471</v>
+        <v>382352.941176471</v>
       </c>
       <c r="M8" s="43" t="inlineStr">
         <is>
@@ -13701,7 +13699,7 @@
       </c>
       <c r="F9" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B9)*D9/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G9" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B9)*D9/$N$18,0)</f>
@@ -13721,7 +13719,7 @@
       </c>
       <c r="K9" s="11">
         <f>OreReserve-SUM($G$6:G9)</f>
-        <v>116470.588235294</v>
+        <v>376470.588235294</v>
       </c>
       <c r="M9" s="43" t="inlineStr">
         <is>
@@ -13754,7 +13752,7 @@
       </c>
       <c r="F10" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B10)*D10/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G10" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B10)*D10/$N$18,0)</f>
@@ -13774,7 +13772,7 @@
       </c>
       <c r="K10" s="11">
         <f>OreReserve-SUM($G$6:G10)</f>
-        <v>110588.235294118</v>
+        <v>370588.235294118</v>
       </c>
       <c r="M10" s="43" t="inlineStr">
         <is>
@@ -13807,7 +13805,7 @@
       </c>
       <c r="F11" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B11)*D11/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G11" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B11)*D11/$N$18,0)</f>
@@ -13827,7 +13825,7 @@
       </c>
       <c r="K11" s="11">
         <f>OreReserve-SUM($G$6:G11)</f>
-        <v>104705.882352941</v>
+        <v>364705.882352941</v>
       </c>
       <c r="M11" s="43" t="inlineStr">
         <is>
@@ -13860,7 +13858,7 @@
       </c>
       <c r="F12" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B12)*D12/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G12" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B12)*D12/$N$18,0)</f>
@@ -13880,7 +13878,7 @@
       </c>
       <c r="K12" s="11">
         <f>OreReserve-SUM($G$6:G12)</f>
-        <v>98823.5294117647</v>
+        <v>358823.529411765</v>
       </c>
       <c r="M12" s="43" t="inlineStr">
         <is>
@@ -13913,7 +13911,7 @@
       </c>
       <c r="F13" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B13)*D13/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G13" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B13)*D13/$N$18,0)</f>
@@ -13933,7 +13931,7 @@
       </c>
       <c r="K13" s="11">
         <f>OreReserve-SUM($G$6:G13)</f>
-        <v>92941.1764705882</v>
+        <v>352941.176470588</v>
       </c>
       <c r="M13" s="43" t="inlineStr">
         <is>
@@ -13966,7 +13964,7 @@
       </c>
       <c r="F14" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B14)*D14/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G14" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B14)*D14/$N$18,0)</f>
@@ -13986,7 +13984,7 @@
       </c>
       <c r="K14" s="11">
         <f>OreReserve-SUM($G$6:G14)</f>
-        <v>87058.8235294118</v>
+        <v>347058.823529412</v>
       </c>
       <c r="M14" s="43" t="inlineStr">
         <is>
@@ -14019,7 +14017,7 @@
       </c>
       <c r="F15" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B15)*D15/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G15" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B15)*D15/$N$18,0)</f>
@@ -14039,7 +14037,7 @@
       </c>
       <c r="K15" s="11">
         <f>OreReserve-SUM($G$6:G15)</f>
-        <v>81176.4705882353</v>
+        <v>341176.470588235</v>
       </c>
       <c r="M15" s="43" t="inlineStr">
         <is>
@@ -14072,7 +14070,7 @@
       </c>
       <c r="F16" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B16)*D16/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G16" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B16)*D16/$N$18,0)</f>
@@ -14092,7 +14090,7 @@
       </c>
       <c r="K16" s="11">
         <f>OreReserve-SUM($G$6:G16)</f>
-        <v>75294.1176470588</v>
+        <v>335294.117647059</v>
       </c>
       <c r="M16" s="43" t="inlineStr">
         <is>
@@ -14125,7 +14123,7 @@
       </c>
       <c r="F17" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B17)*D17/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G17" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B17)*D17/$N$18,0)</f>
@@ -14145,7 +14143,7 @@
       </c>
       <c r="K17" s="11">
         <f>OreReserve-SUM($G$6:G17)</f>
-        <v>69411.7647058824</v>
+        <v>329411.764705882</v>
       </c>
       <c r="M17" s="43" t="inlineStr">
         <is>
@@ -14178,7 +14176,7 @@
       </c>
       <c r="F18" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B18)*D18/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G18" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B18)*D18/$N$18,0)</f>
@@ -14198,7 +14196,7 @@
       </c>
       <c r="K18" s="11">
         <f>OreReserve-SUM($G$6:G18)</f>
-        <v>63529.4117647059</v>
+        <v>323529.411764706</v>
       </c>
       <c r="M18" s="32" t="inlineStr">
         <is>
@@ -14232,7 +14230,7 @@
       </c>
       <c r="F19" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B19)*D19/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G19" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B19)*D19/$N$18,0)</f>
@@ -14252,7 +14250,7 @@
       </c>
       <c r="K19" s="11">
         <f>OreReserve-SUM($G$6:G19)</f>
-        <v>57647.0588235294</v>
+        <v>317647.058823529</v>
       </c>
       <c r="M19" s="43" t="inlineStr">
         <is>
@@ -14286,7 +14284,7 @@
       </c>
       <c r="F20" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B20)*D20/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G20" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B20)*D20/$N$18,0)</f>
@@ -14306,7 +14304,7 @@
       </c>
       <c r="K20" s="11">
         <f>OreReserve-SUM($G$6:G20)</f>
-        <v>51764.7058823529</v>
+        <v>311764.705882353</v>
       </c>
       <c r="M20" s="43" t="inlineStr">
         <is>
@@ -14340,7 +14338,7 @@
       </c>
       <c r="F21" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B21)*D21/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G21" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B21)*D21/$N$18,0)</f>
@@ -14360,7 +14358,7 @@
       </c>
       <c r="K21" s="11">
         <f>OreReserve-SUM($G$6:G21)</f>
-        <v>45882.3529411765</v>
+        <v>305882.352941177</v>
       </c>
       <c r="M21" s="43" t="inlineStr">
         <is>
@@ -14394,7 +14392,7 @@
       </c>
       <c r="F22" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B22)*D22/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G22" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B22)*D22/$N$18,0)</f>
@@ -14414,7 +14412,7 @@
       </c>
       <c r="K22" s="11">
         <f>OreReserve-SUM($G$6:G22)</f>
-        <v>40000</v>
+        <v>300000</v>
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
@@ -14444,7 +14442,7 @@
       </c>
       <c r="F23" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B23)*D23/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G23" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B23)*D23/$N$18,0)</f>
@@ -14464,7 +14462,7 @@
       </c>
       <c r="K23" s="11">
         <f>OreReserve-SUM($G$6:G23)</f>
-        <v>34117.6470588235</v>
+        <v>294117.647058824</v>
       </c>
     </row>
     <row r="24">
@@ -14489,7 +14487,7 @@
       </c>
       <c r="F24" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B24)*D24/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G24" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B24)*D24/$N$18,0)</f>
@@ -14509,7 +14507,7 @@
       </c>
       <c r="K24" s="11">
         <f>OreReserve-SUM($G$6:G24)</f>
-        <v>28235.2941176471</v>
+        <v>288235.294117647</v>
       </c>
       <c r="M24" s="15" t="inlineStr">
         <is>
@@ -14542,7 +14540,7 @@
       </c>
       <c r="F25" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B25)*D25/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G25" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B25)*D25/$N$18,0)</f>
@@ -14562,7 +14560,7 @@
       </c>
       <c r="K25" s="11">
         <f>OreReserve-SUM($G$6:G25)</f>
-        <v>22352.9411764706</v>
+        <v>282352.941176471</v>
       </c>
       <c r="M25" s="6" t="inlineStr">
         <is>
@@ -14607,7 +14605,7 @@
       </c>
       <c r="F26" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B26)*D26/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G26" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B26)*D26/$N$18,0)</f>
@@ -14627,7 +14625,7 @@
       </c>
       <c r="K26" s="11">
         <f>OreReserve-SUM($G$6:G26)</f>
-        <v>16470.5882352941</v>
+        <v>276470.588235294</v>
       </c>
       <c r="M26" s="7" t="n">
         <v>1</v>
@@ -14667,7 +14665,7 @@
       </c>
       <c r="F27" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B27)*D27/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G27" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B27)*D27/$N$18,0)</f>
@@ -14687,7 +14685,7 @@
       </c>
       <c r="K27" s="11">
         <f>OreReserve-SUM($G$6:G27)</f>
-        <v>10588.2352941177</v>
+        <v>270588.235294118</v>
       </c>
       <c r="M27" s="7" t="n">
         <v>2</v>
@@ -14727,7 +14725,7 @@
       </c>
       <c r="F28" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B28)*D28/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G28" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B28)*D28/$N$18,0)</f>
@@ -14747,7 +14745,7 @@
       </c>
       <c r="K28" s="11">
         <f>OreReserve-SUM($G$6:G28)</f>
-        <v>4705.88235294118</v>
+        <v>264705.882352941</v>
       </c>
       <c r="M28" s="7" t="n">
         <v>3</v>
@@ -14787,7 +14785,7 @@
       </c>
       <c r="F29" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B29)*D29/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G29" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B29)*D29/$N$18,0)</f>
@@ -14807,7 +14805,7 @@
       </c>
       <c r="K29" s="11">
         <f>OreReserve-SUM($G$6:G29)</f>
-        <v>-1176.4705882353</v>
+        <v>258823.529411765</v>
       </c>
       <c r="M29" s="7" t="n">
         <v>4</v>
@@ -14847,7 +14845,7 @@
       </c>
       <c r="F30" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B30)*D30/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G30" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B30)*D30/$N$18,0)</f>
@@ -14867,7 +14865,7 @@
       </c>
       <c r="K30" s="11">
         <f>OreReserve-SUM($G$6:G30)</f>
-        <v>-7058.82352941178</v>
+        <v>252941.176470588</v>
       </c>
       <c r="M30" s="7" t="n">
         <v>5</v>
@@ -14907,7 +14905,7 @@
       </c>
       <c r="F31" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B31)*D31/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G31" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B31)*D31/$N$18,0)</f>
@@ -14927,7 +14925,7 @@
       </c>
       <c r="K31" s="11">
         <f>OreReserve-SUM($G$6:G31)</f>
-        <v>-12941.1764705882</v>
+        <v>247058.823529412</v>
       </c>
       <c r="M31" s="32" t="inlineStr">
         <is>
@@ -14969,7 +14967,7 @@
       </c>
       <c r="F32" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B32)*D32/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G32" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B32)*D32/$N$18,0)</f>
@@ -14989,7 +14987,7 @@
       </c>
       <c r="K32" s="11">
         <f>OreReserve-SUM($G$6:G32)</f>
-        <v>-18823.5294117647</v>
+        <v>241176.470588235</v>
       </c>
       <c r="M32" s="32" t="inlineStr">
         <is>
@@ -15023,7 +15021,7 @@
       </c>
       <c r="F33" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B33)*D33/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G33" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B33)*D33/$N$18,0)</f>
@@ -15043,7 +15041,7 @@
       </c>
       <c r="K33" s="11">
         <f>OreReserve-SUM($G$6:G33)</f>
-        <v>-24705.8823529412</v>
+        <v>235294.117647059</v>
       </c>
     </row>
     <row r="34">
@@ -15068,7 +15066,7 @@
       </c>
       <c r="F34" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B34)*D34/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G34" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B34)*D34/$N$18,0)</f>
@@ -15088,7 +15086,7 @@
       </c>
       <c r="K34" s="11">
         <f>OreReserve-SUM($G$6:G34)</f>
-        <v>-30588.2352941177</v>
+        <v>229411.764705882</v>
       </c>
     </row>
     <row r="35">
@@ -15113,7 +15111,7 @@
       </c>
       <c r="F35" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B35)*D35/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G35" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B35)*D35/$N$18,0)</f>
@@ -15133,7 +15131,7 @@
       </c>
       <c r="K35" s="11">
         <f>OreReserve-SUM($G$6:G35)</f>
-        <v>-36470.5882352941</v>
+        <v>223529.411764706</v>
       </c>
     </row>
     <row r="36">
@@ -15158,7 +15156,7 @@
       </c>
       <c r="F36" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B36)*D36/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G36" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B36)*D36/$N$18,0)</f>
@@ -15178,7 +15176,7 @@
       </c>
       <c r="K36" s="11">
         <f>OreReserve-SUM($G$6:G36)</f>
-        <v>-42352.9411764706</v>
+        <v>217647.058823529</v>
       </c>
     </row>
     <row r="37">
@@ -15203,7 +15201,7 @@
       </c>
       <c r="F37" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B37)*D37/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G37" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B37)*D37/$N$18,0)</f>
@@ -15223,7 +15221,7 @@
       </c>
       <c r="K37" s="11">
         <f>OreReserve-SUM($G$6:G37)</f>
-        <v>-48235.2941176471</v>
+        <v>211764.705882353</v>
       </c>
     </row>
     <row r="38">
@@ -15248,7 +15246,7 @@
       </c>
       <c r="F38" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B38)*D38/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G38" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B38)*D38/$N$18,0)</f>
@@ -15268,7 +15266,7 @@
       </c>
       <c r="K38" s="11">
         <f>OreReserve-SUM($G$6:G38)</f>
-        <v>-54117.6470588235</v>
+        <v>205882.352941176</v>
       </c>
     </row>
     <row r="39">
@@ -15293,7 +15291,7 @@
       </c>
       <c r="F39" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B39)*D39/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G39" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B39)*D39/$N$18,0)</f>
@@ -15313,7 +15311,7 @@
       </c>
       <c r="K39" s="11">
         <f>OreReserve-SUM($G$6:G39)</f>
-        <v>-60000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="40">
@@ -15338,7 +15336,7 @@
       </c>
       <c r="F40" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B40)*D40/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G40" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B40)*D40/$N$18,0)</f>
@@ -15358,7 +15356,7 @@
       </c>
       <c r="K40" s="11">
         <f>OreReserve-SUM($G$6:G40)</f>
-        <v>-65882.3529411765</v>
+        <v>194117.647058824</v>
       </c>
     </row>
     <row r="41">
@@ -15383,7 +15381,7 @@
       </c>
       <c r="F41" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B41)*D41/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G41" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B41)*D41/$N$18,0)</f>
@@ -15403,7 +15401,7 @@
       </c>
       <c r="K41" s="11">
         <f>OreReserve-SUM($G$6:G41)</f>
-        <v>-71764.7058823529</v>
+        <v>188235.294117647</v>
       </c>
     </row>
     <row r="42">
@@ -15428,7 +15426,7 @@
       </c>
       <c r="F42" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B42)*D42/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G42" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B42)*D42/$N$18,0)</f>
@@ -15448,7 +15446,7 @@
       </c>
       <c r="K42" s="11">
         <f>OreReserve-SUM($G$6:G42)</f>
-        <v>-77647.0588235294</v>
+        <v>182352.941176471</v>
       </c>
     </row>
     <row r="43">
@@ -15473,7 +15471,7 @@
       </c>
       <c r="F43" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B43)*D43/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G43" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B43)*D43/$N$18,0)</f>
@@ -15493,7 +15491,7 @@
       </c>
       <c r="K43" s="11">
         <f>OreReserve-SUM($G$6:G43)</f>
-        <v>-83529.4117647059</v>
+        <v>176470.588235294</v>
       </c>
     </row>
     <row r="44">
@@ -15518,7 +15516,7 @@
       </c>
       <c r="F44" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B44)*D44/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G44" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B44)*D44/$N$18,0)</f>
@@ -15538,7 +15536,7 @@
       </c>
       <c r="K44" s="11">
         <f>OreReserve-SUM($G$6:G44)</f>
-        <v>-89411.7647058824</v>
+        <v>170588.235294118</v>
       </c>
     </row>
     <row r="45">
@@ -15563,7 +15561,7 @@
       </c>
       <c r="F45" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B45)*D45/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G45" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B45)*D45/$N$18,0)</f>
@@ -15583,7 +15581,7 @@
       </c>
       <c r="K45" s="11">
         <f>OreReserve-SUM($G$6:G45)</f>
-        <v>-95294.1176470588</v>
+        <v>164705.882352941</v>
       </c>
     </row>
     <row r="46">
@@ -15608,7 +15606,7 @@
       </c>
       <c r="F46" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B46)*D46/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G46" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B46)*D46/$N$18,0)</f>
@@ -15628,7 +15626,7 @@
       </c>
       <c r="K46" s="11">
         <f>OreReserve-SUM($G$6:G46)</f>
-        <v>-101176.470588235</v>
+        <v>158823.529411765</v>
       </c>
     </row>
     <row r="47">
@@ -15653,7 +15651,7 @@
       </c>
       <c r="F47" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B47)*D47/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G47" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B47)*D47/$N$18,0)</f>
@@ -15673,7 +15671,7 @@
       </c>
       <c r="K47" s="11">
         <f>OreReserve-SUM($G$6:G47)</f>
-        <v>-107058.823529412</v>
+        <v>152941.176470588</v>
       </c>
     </row>
     <row r="48">
@@ -15698,7 +15696,7 @@
       </c>
       <c r="F48" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B48)*D48/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G48" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B48)*D48/$N$18,0)</f>
@@ -15718,7 +15716,7 @@
       </c>
       <c r="K48" s="11">
         <f>OreReserve-SUM($G$6:G48)</f>
-        <v>-112941.176470588</v>
+        <v>147058.823529412</v>
       </c>
     </row>
     <row r="49">
@@ -15743,7 +15741,7 @@
       </c>
       <c r="F49" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B49)*D49/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G49" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B49)*D49/$N$18,0)</f>
@@ -15763,7 +15761,7 @@
       </c>
       <c r="K49" s="11">
         <f>OreReserve-SUM($G$6:G49)</f>
-        <v>-118823.529411765</v>
+        <v>141176.470588235</v>
       </c>
     </row>
     <row r="50">
@@ -15788,7 +15786,7 @@
       </c>
       <c r="F50" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B50)*D50/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G50" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B50)*D50/$N$18,0)</f>
@@ -15808,7 +15806,7 @@
       </c>
       <c r="K50" s="11">
         <f>OreReserve-SUM($G$6:G50)</f>
-        <v>-124705.882352941</v>
+        <v>135294.117647059</v>
       </c>
     </row>
     <row r="51">
@@ -15833,7 +15831,7 @@
       </c>
       <c r="F51" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B51)*D51/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G51" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B51)*D51/$N$18,0)</f>
@@ -15853,7 +15851,7 @@
       </c>
       <c r="K51" s="11">
         <f>OreReserve-SUM($G$6:G51)</f>
-        <v>-130588.235294118</v>
+        <v>129411.764705882</v>
       </c>
     </row>
     <row r="52">
@@ -15878,7 +15876,7 @@
       </c>
       <c r="F52" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B52)*D52/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G52" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B52)*D52/$N$18,0)</f>
@@ -15898,7 +15896,7 @@
       </c>
       <c r="K52" s="11">
         <f>OreReserve-SUM($G$6:G52)</f>
-        <v>-136470.588235294</v>
+        <v>123529.411764706</v>
       </c>
     </row>
     <row r="53">
@@ -15923,7 +15921,7 @@
       </c>
       <c r="F53" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B53)*D53/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G53" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B53)*D53/$N$18,0)</f>
@@ -15943,7 +15941,7 @@
       </c>
       <c r="K53" s="11">
         <f>OreReserve-SUM($G$6:G53)</f>
-        <v>-142352.941176471</v>
+        <v>117647.058823529</v>
       </c>
     </row>
     <row r="54">
@@ -15968,7 +15966,7 @@
       </c>
       <c r="F54" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B54)*D54/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G54" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B54)*D54/$N$18,0)</f>
@@ -15988,7 +15986,7 @@
       </c>
       <c r="K54" s="11">
         <f>OreReserve-SUM($G$6:G54)</f>
-        <v>-148235.294117647</v>
+        <v>111764.705882353</v>
       </c>
     </row>
     <row r="55">
@@ -16013,7 +16011,7 @@
       </c>
       <c r="F55" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B55)*D55/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G55" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B55)*D55/$N$18,0)</f>
@@ -16033,7 +16031,7 @@
       </c>
       <c r="K55" s="11">
         <f>OreReserve-SUM($G$6:G55)</f>
-        <v>-154117.647058824</v>
+        <v>105882.352941177</v>
       </c>
     </row>
     <row r="56">
@@ -16058,7 +16056,7 @@
       </c>
       <c r="F56" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B56)*D56/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G56" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B56)*D56/$N$18,0)</f>
@@ -16078,7 +16076,7 @@
       </c>
       <c r="K56" s="11">
         <f>OreReserve-SUM($G$6:G56)</f>
-        <v>-160000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="57">
@@ -16103,7 +16101,7 @@
       </c>
       <c r="F57" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B57)*D57/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G57" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B57)*D57/$N$18,0)</f>
@@ -16123,7 +16121,7 @@
       </c>
       <c r="K57" s="11">
         <f>OreReserve-SUM($G$6:G57)</f>
-        <v>-165882.352941176</v>
+        <v>94117.6470588236</v>
       </c>
     </row>
     <row r="58">
@@ -16148,7 +16146,7 @@
       </c>
       <c r="F58" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B58)*D58/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G58" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B58)*D58/$N$18,0)</f>
@@ -16168,7 +16166,7 @@
       </c>
       <c r="K58" s="11">
         <f>OreReserve-SUM($G$6:G58)</f>
-        <v>-171764.705882353</v>
+        <v>88235.2941176471</v>
       </c>
     </row>
     <row r="59">
@@ -16193,7 +16191,7 @@
       </c>
       <c r="F59" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B59)*D59/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G59" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B59)*D59/$N$18,0)</f>
@@ -16213,7 +16211,7 @@
       </c>
       <c r="K59" s="11">
         <f>OreReserve-SUM($G$6:G59)</f>
-        <v>-177647.058823529</v>
+        <v>82352.9411764706</v>
       </c>
     </row>
     <row r="60">
@@ -16238,7 +16236,7 @@
       </c>
       <c r="F60" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B60)*D60/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G60" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B60)*D60/$N$18,0)</f>
@@ -16258,7 +16256,7 @@
       </c>
       <c r="K60" s="11">
         <f>OreReserve-SUM($G$6:G60)</f>
-        <v>-183529.411764706</v>
+        <v>76470.5882352942</v>
       </c>
     </row>
     <row r="61">
@@ -16283,7 +16281,7 @@
       </c>
       <c r="F61" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B61)*D61/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G61" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B61)*D61/$N$18,0)</f>
@@ -16303,7 +16301,7 @@
       </c>
       <c r="K61" s="11">
         <f>OreReserve-SUM($G$6:G61)</f>
-        <v>-189411.764705882</v>
+        <v>70588.2352941177</v>
       </c>
     </row>
     <row r="62">
@@ -16328,7 +16326,7 @@
       </c>
       <c r="F62" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B62)*D62/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G62" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B62)*D62/$N$18,0)</f>
@@ -16348,7 +16346,7 @@
       </c>
       <c r="K62" s="11">
         <f>OreReserve-SUM($G$6:G62)</f>
-        <v>-195294.117647059</v>
+        <v>64705.8823529412</v>
       </c>
     </row>
     <row r="63">
@@ -16373,7 +16371,7 @@
       </c>
       <c r="F63" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B63)*D63/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G63" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B63)*D63/$N$18,0)</f>
@@ -16393,7 +16391,7 @@
       </c>
       <c r="K63" s="11">
         <f>OreReserve-SUM($G$6:G63)</f>
-        <v>-201176.470588235</v>
+        <v>58823.5294117648</v>
       </c>
     </row>
     <row r="64">
@@ -16418,7 +16416,7 @@
       </c>
       <c r="F64" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B64)*D64/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G64" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B64)*D64/$N$18,0)</f>
@@ -16438,7 +16436,7 @@
       </c>
       <c r="K64" s="11">
         <f>OreReserve-SUM($G$6:G64)</f>
-        <v>-207058.823529412</v>
+        <v>52941.1764705883</v>
       </c>
     </row>
     <row r="65">
@@ -16463,7 +16461,7 @@
       </c>
       <c r="F65" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$22:$H$22,B65)*D65/$N$18,0)</f>
-        <v>52941.1764705882</v>
+        <v>29411.7647058824</v>
       </c>
       <c r="G65" s="11">
         <f>IF($N$18&gt;0,INDEX('الخطة الفنية والإنتاج'!$D$23:$H$23,B65)*D65/$N$18,0)</f>
@@ -16483,7 +16481,7 @@
       </c>
       <c r="K65" s="11">
         <f>OreReserve-SUM($G$6:G65)</f>
-        <v>-212941.176470588</v>
+        <v>47058.8235294118</v>
       </c>
     </row>
     <row r="66">
@@ -16501,7 +16499,7 @@
       <c r="E66" s="12" t="n"/>
       <c r="F66" s="12">
         <f>SUM(F6:F65)</f>
-        <v>3176470.58823529</v>
+        <v>1764705.88235294</v>
       </c>
       <c r="G66" s="12">
         <f>SUM(G6:G65)</f>

</xml_diff>